<commit_message>
Plan de compras: el simulador arranca del conteo fisico por camara
Correccion: el conteo del 17/09 (conteo-todas-2026-09-18.xlsx) estaba en
Descargas y se habia ignorado; el "Stock" del reporte diario del ERP es
solo lo listo para vender ese dia, no la camara. Ahora:
- fuentes/stock/2026-09-17_conteo_camaras.xlsx (el archivo tal cual).
- plan_compras.xlsx: hoja 'conteo' (fecha, origen, cajas): BR 14.475,
  PY 12.345, BO 2.604, EC 23.654 de referencia; notas actualizadas.
- plan_compras.json: bloque conteo y descarga_est por camion.
- index_compras.html: tarjeta "Conteo fisico (arranque)" editable (fecha
  y cajas por origen) en vez de "colchon inicial"; el saldo parte del
  conteo y solo suma los camiones que descargan despues de esa fecha; la
  semana del conteo prorratea la venta por los dias que quedan.

Verificado con una replica en PowerShell de la misma regla.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/plan_compras.xlsx
+++ b/fuentes/plan_compras.xlsx
@@ -8,13 +8,14 @@
     <sheet name="cargas_programadas" sheetId="1" r:id="rId1"/>
     <sheet name="ventas_plan" sheetId="2" r:id="rId3"/>
     <sheet name="notas" sheetId="3" r:id="rId4"/>
+    <sheet name="conteo" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>fecha</t>
   </si>
@@ -176,6 +177,30 @@
   </si>
   <si>
     <t>Historial: 19/09/2026 creado con las semanas 14-19/09 (real) y 21-26/09 (programada) dictadas por Gonzalo.</t>
+  </si>
+  <si>
+    <t>5. conteo: stock fisico de banana por origen (cajas) a la fecha del conteo por camara (todas las sedes). El simulador ARRANCA de este numero: suma los camiones que descargan despues de esa fecha y resta la venta. Cada conteo nuevo es una fila mas; se usa el mas reciente. El "Stock" del reporte diario del ERP NO es esto: es solo la fruta lista para vender ese dia.</t>
+  </si>
+  <si>
+    <t>Historial: 19/09/2026 hoja conteo con el conteo del 17/09 (BR 14.475, PY 12.345, BO 2.604).</t>
+  </si>
+  <si>
+    <t>fuentes\stock\2026-09-17_conteo_camaras.xlsx</t>
+  </si>
+  <si>
+    <t>ZAC 13.467 + Coronel Raiz 1.008; sin palta ni mandioca</t>
+  </si>
+  <si>
+    <t>ZAC 9.402 + Coronel Raiz 2.943</t>
+  </si>
+  <si>
+    <t>ZAC camaras 18, 25 y 29 (Porvenir)</t>
+  </si>
+  <si>
+    <t>EC</t>
+  </si>
+  <si>
+    <t>referencia; Ecuador no entra en el plan</t>
   </si>
 </sst>
 </file>
@@ -214,8 +239,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
@@ -1210,7 +1237,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="218.08561706543" customWidth="1"/>
@@ -1256,6 +1283,118 @@
         <v>53</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" customWidth="1"/>
+    <col min="4" max="4" width="43.748161315918" customWidth="1"/>
+    <col min="5" max="5" width="49.3576278686523" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5">
+        <v>46282</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="0">
+        <v>14475</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5">
+        <v>46282</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="0">
+        <v>12345</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5">
+        <v>46282</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="0">
+        <v>2604</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5">
+        <v>46282</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="0">
+        <v>23654</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>61</v>
+      </c>
+    </row>
   </sheetData>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
Stock ERP del 16/09 y 19/09, ventas diarias fechadas, y el simulador los muestra
- fuentes/stock/2026-09-19_stock_erp_captura.jpeg (reporte del sabado al
  cierre) y filas del 16/09 y 19/09 en stock_diario.xlsx (el 16/09 estaba
  como captura pero no cargado). Stock = fruta lista para vender.
- plan_compras.xlsx: hoja ventas_erp con las cajas vendidas por dia y
  origen de los reportes fechados (15, 16 y 19/09) para calibrar
  ventas_plan; nota en la hoja notas.
- plan_compras.json: bloque stock_erp (ultimo dia de stock_diario);
  index_compras.html lo muestra en la tarjeta de cada origen ("listo
  para vender al 19/09").

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/plan_compras.xlsx
+++ b/fuentes/plan_compras.xlsx
@@ -9,13 +9,14 @@
     <sheet name="ventas_plan" sheetId="2" r:id="rId3"/>
     <sheet name="notas" sheetId="3" r:id="rId4"/>
     <sheet name="conteo" sheetId="4" r:id="rId5"/>
+    <sheet name="ventas_erp" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
   <si>
     <t>fecha</t>
   </si>
@@ -185,6 +186,9 @@
     <t>Historial: 19/09/2026 hoja conteo con el conteo del 17/09 (BR 14.475, PY 12.345, BO 2.604).</t>
   </si>
   <si>
+    <t>6. ventas_erp: cajas vendidas por dia y origen segun el reporte diario del ERP (columna Present. = cajas, Kilos = kg; Stock = kg listos para vender ese dia, NO la camara). Sirve para calibrar ventas_plan. Hay un reporte mas de la semana 38 (5.750 cajas, dia fuerte) sin fecha: no se cargo.</t>
+  </si>
+  <si>
     <t>fuentes\stock\2026-09-17_conteo_camaras.xlsx</t>
   </si>
   <si>
@@ -201,6 +205,24 @@
   </si>
   <si>
     <t>referencia; Ecuador no entra en el plan</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>stock_listo_kg</t>
+  </si>
+  <si>
+    <t>reporte ERP 15/09</t>
+  </si>
+  <si>
+    <t>mie</t>
+  </si>
+  <si>
+    <t>reporte ERP 16/09</t>
+  </si>
+  <si>
+    <t>reporte ERP 19/09 cierre</t>
   </si>
 </sst>
 </file>
@@ -239,8 +261,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="22" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0" applyProtection="1"/>
@@ -1237,7 +1261,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="218.08561706543" customWidth="1"/>
@@ -1291,6 +1315,11 @@
     <row r="10">
       <c r="A10" s="0" t="s">
         <v>55</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1338,10 +1367,10 @@
         <v>14475</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3">
@@ -1355,10 +1384,10 @@
         <v>12345</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
@@ -1372,10 +1401,10 @@
         <v>2604</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5">
@@ -1383,16 +1412,334 @@
         <v>46282</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C5" s="0">
         <v>23654</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E5" s="0" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.8945598602295" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" customWidth="1"/>
+    <col min="6" max="6" width="14.159068107605" customWidth="1"/>
+    <col min="7" max="7" width="23.1323738098145" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7">
+        <v>46280</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="0">
+        <v>964</v>
+      </c>
+      <c r="E2" s="0">
+        <v>21208</v>
+      </c>
+      <c r="F2" s="0">
+        <v>21026</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7">
+        <v>46280</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="0">
+        <v>725</v>
+      </c>
+      <c r="E3" s="0">
+        <v>15950</v>
+      </c>
+      <c r="F3" s="0">
+        <v>10628</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7">
+        <v>46280</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="0">
+        <v>98</v>
+      </c>
+      <c r="E4" s="0">
+        <v>1960</v>
+      </c>
+      <c r="F4" s="0">
+        <v>1958</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7">
+        <v>46280</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="0" t="s">
         <v>61</v>
+      </c>
+      <c r="D5" s="0">
+        <v>996</v>
+      </c>
+      <c r="E5" s="0">
+        <v>18924</v>
+      </c>
+      <c r="F5" s="0">
+        <v>23023</v>
+      </c>
+      <c r="G5" s="0" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7">
+        <v>46281</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="0">
+        <v>1301</v>
+      </c>
+      <c r="E6" s="0">
+        <v>28622</v>
+      </c>
+      <c r="F6" s="0">
+        <v>19725</v>
+      </c>
+      <c r="G6" s="0" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7">
+        <v>46281</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="0">
+        <v>710</v>
+      </c>
+      <c r="E7" s="0">
+        <v>15620</v>
+      </c>
+      <c r="F7" s="0">
+        <v>11881</v>
+      </c>
+      <c r="G7" s="0" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7">
+        <v>46281</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="0">
+        <v>114</v>
+      </c>
+      <c r="E8" s="0">
+        <v>2280</v>
+      </c>
+      <c r="F8" s="0">
+        <v>1844</v>
+      </c>
+      <c r="G8" s="0" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7">
+        <v>46281</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="D9" s="0">
+        <v>942</v>
+      </c>
+      <c r="E9" s="0">
+        <v>17898</v>
+      </c>
+      <c r="F9" s="0">
+        <v>22081</v>
+      </c>
+      <c r="G9" s="0" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7">
+        <v>46284</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="0">
+        <v>749</v>
+      </c>
+      <c r="E10" s="0">
+        <v>16478</v>
+      </c>
+      <c r="F10" s="0">
+        <v>15893</v>
+      </c>
+      <c r="G10" s="0" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7">
+        <v>46284</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="0">
+        <v>686</v>
+      </c>
+      <c r="E11" s="0">
+        <v>15092</v>
+      </c>
+      <c r="F11" s="0">
+        <v>14132</v>
+      </c>
+      <c r="G11" s="0" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7">
+        <v>46284</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="0">
+        <v>139</v>
+      </c>
+      <c r="E12" s="0">
+        <v>2780</v>
+      </c>
+      <c r="F12" s="0">
+        <v>1972</v>
+      </c>
+      <c r="G12" s="0" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7">
+        <v>46284</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="D13" s="0">
+        <v>832</v>
+      </c>
+      <c r="E13" s="0">
+        <v>15808</v>
+      </c>
+      <c r="F13" s="0">
+        <v>20033</v>
+      </c>
+      <c r="G13" s="0" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>